<commit_message>
Reproduce disease-context table and synchronize all manuscript outputs
</commit_message>
<xml_diff>
--- a/tables/Main_Tables.xlsx
+++ b/tables/Main_Tables.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table1'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table2'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table2'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Table3'!$A$1:$G$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -596,16 +598,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Record or disease annotation</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Records</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence in the fixed export</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>USH2A VariationID 2353; Usher syndrome among its annotations</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pathogenic; 3 review stars (expert panel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CFTR records; cystic fibrosis among every record’s annotations</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Pathogenic; 4 review stars (practice guideline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Familial isolated dilated cardiomyopathy (ORPHA:154)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>44,036</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Matching disease identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Primary ciliary dyskinesia (ORPHA:244)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>28,729</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Matching disease identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fanconi anemia (ORPHA:84)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>27,050</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Matching disease identifier</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -641,7 +765,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Other/unknown</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
@@ -715,8 +839,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>3</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>3: expert panel</t>
+        </is>
       </c>
       <c r="B5" s="2" t="n">
         <v>173</v>
@@ -738,8 +864,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>4</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>4: practice guideline</t>
+        </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>0</v>

</xml_diff>